<commit_message>
Add screenshots for reports and CI validation
</commit_message>
<xml_diff>
--- a/testData/DeleteOrder.xlsx
+++ b/testData/DeleteOrder.xlsx
@@ -14,18 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>orderId</t>
   </si>
   <si>
     <t>expectedStatus</t>
-  </si>
-  <si>
-    <t>abc</t>
-  </si>
-  <si>
-    <t>@@@</t>
   </si>
 </sst>
 </file>
@@ -381,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="20.77734375" customWidth="1"/>
@@ -443,22 +437,6 @@
         <v>404</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="2">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="2">
-        <v>400</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>